<commit_message>
Update meetings and reminders spreadsheets
</commit_message>
<xml_diff>
--- a/meetings.xlsx
+++ b/meetings.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sivane\Desktop\ai-dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AC37959-E689-416B-9445-ACCC978E129C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABBF41A7-AD30-4743-B13B-8C7C01069974}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20" yWindow="20" windowWidth="19180" windowHeight="10060" xr2:uid="{654D42B8-71DE-4F6E-86CF-583F17BFBCF2}"/>
+    <workbookView xWindow="20" yWindow="740" windowWidth="19180" windowHeight="10060" xr2:uid="{654D42B8-71DE-4F6E-86CF-583F17BFBCF2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="15">
   <si>
     <t>project_name</t>
   </si>
@@ -75,6 +75,12 @@
   </si>
   <si>
     <t>פרויקט אישי - דשבורד</t>
+  </si>
+  <si>
+    <t xml:space="preserve">בנק יהב </t>
+  </si>
+  <si>
+    <t>מעבר על ליקויי אבטחה</t>
   </si>
 </sst>
 </file>
@@ -468,7 +474,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81840B73-A939-4138-9F05-60B93E3DBEB3}">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultColWidth="8.08203125" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.5" customWidth="1"/>
@@ -507,7 +513,7 @@
         <v>6</v>
       </c>
       <c r="C2" s="3">
-        <v>46129</v>
+        <v>46131</v>
       </c>
       <c r="D2" s="4">
         <v>0.41666666666666669</v>
@@ -527,7 +533,7 @@
         <v>9</v>
       </c>
       <c r="C3" s="3">
-        <v>46129</v>
+        <v>46131</v>
       </c>
       <c r="D3" s="4">
         <v>0.60416666666666663</v>
@@ -536,6 +542,26 @@
         <v>10</v>
       </c>
       <c r="F3" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" s="3">
+        <v>46131</v>
+      </c>
+      <c r="D4" s="4">
+        <v>0.64583333333333337</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" s="2" t="s">
         <v>8</v>
       </c>
     </row>

</xml_diff>

<commit_message>
updated meetings.xlsx with start_time and End_time columns
</commit_message>
<xml_diff>
--- a/meetings.xlsx
+++ b/meetings.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sivane\Desktop\ai-dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABBF41A7-AD30-4743-B13B-8C7C01069974}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{347EC3FB-1B72-4243-9EBD-6BA1BE9F0BF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20" yWindow="740" windowWidth="19180" windowHeight="10060" xr2:uid="{654D42B8-71DE-4F6E-86CF-583F17BFBCF2}"/>
+    <workbookView xWindow="20" yWindow="20" windowWidth="19180" windowHeight="10060" xr2:uid="{654D42B8-71DE-4F6E-86CF-583F17BFBCF2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="16">
   <si>
     <t>project_name</t>
   </si>
@@ -47,9 +47,6 @@
     <t>date</t>
   </si>
   <si>
-    <t>time</t>
-  </si>
-  <si>
     <t>owner</t>
   </si>
   <si>
@@ -81,6 +78,12 @@
   </si>
   <si>
     <t>מעבר על ליקויי אבטחה</t>
+  </si>
+  <si>
+    <t>start_time</t>
+  </si>
+  <si>
+    <t>end_time</t>
   </si>
 </sst>
 </file>
@@ -474,18 +477,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{81840B73-A939-4138-9F05-60B93E3DBEB3}">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr defaultColWidth="8.08203125" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.5" customWidth="1"/>
     <col min="2" max="2" width="19.1640625" customWidth="1"/>
     <col min="3" max="3" width="18.1640625" customWidth="1"/>
-    <col min="4" max="4" width="12.25" customWidth="1"/>
-    <col min="5" max="5" width="13" customWidth="1"/>
-    <col min="6" max="6" width="12.1640625" customWidth="1"/>
+    <col min="4" max="5" width="12.25" customWidth="1"/>
+    <col min="6" max="6" width="13" customWidth="1"/>
+    <col min="7" max="7" width="12.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="28" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -496,21 +499,24 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>6</v>
       </c>
       <c r="C2" s="3">
         <v>46131</v>
@@ -518,19 +524,22 @@
       <c r="D2" s="4">
         <v>0.41666666666666669</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="4">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F2" s="2" t="s">
+    </row>
+    <row r="3" spans="1:7" ht="28" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" ht="28" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>9</v>
       </c>
       <c r="C3" s="3">
         <v>46131</v>
@@ -538,19 +547,22 @@
       <c r="D3" s="4">
         <v>0.60416666666666663</v>
       </c>
-      <c r="E3" s="2" t="s">
-        <v>10</v>
+      <c r="E3" s="4">
+        <v>0.625</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>13</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>14</v>
       </c>
       <c r="C4" s="3">
         <v>46131</v>
@@ -558,11 +570,14 @@
       <c r="D4" s="4">
         <v>0.64583333333333337</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="4">
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G4" s="2" t="s">
         <v>7</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>